<commit_message>
update news midtown & avenue
</commit_message>
<xml_diff>
--- a/public/documents/k-home-avenue-80-bai-seo.xlsx
+++ b/public/documents/k-home-avenue-80-bai-seo.xlsx
@@ -560,7 +560,7 @@
         <v>Chính sách</v>
       </c>
       <c r="G7" t="str">
-        <v/>
+        <v>Done</v>
       </c>
     </row>
     <row r="8">
@@ -583,7 +583,7 @@
         <v>Chính sách</v>
       </c>
       <c r="G8" t="str">
-        <v/>
+        <v>Done</v>
       </c>
     </row>
     <row r="9">
@@ -606,7 +606,7 @@
         <v>Chính sách</v>
       </c>
       <c r="G9" t="str">
-        <v/>
+        <v>Done</v>
       </c>
     </row>
     <row r="10">
@@ -629,7 +629,7 @@
         <v>Đánh giá dự án</v>
       </c>
       <c r="G10" t="str">
-        <v/>
+        <v>Done</v>
       </c>
     </row>
     <row r="11">
@@ -652,7 +652,7 @@
         <v>Chính sách</v>
       </c>
       <c r="G11" t="str">
-        <v/>
+        <v>Done</v>
       </c>
     </row>
     <row r="12">

</xml_diff>